<commit_message>
Add link of BOE2
</commit_message>
<xml_diff>
--- a/data/RSS_link.xlsx
+++ b/data/RSS_link.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8779c4def3e22337/ドキュメント/GitHub/rss-daily-digest/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="69" documentId="11_AD4D066CA252ABDACC10489A1917CC5073EEDF52" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D65D411E-2735-44D6-B862-EF0795D23A9B}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="11_AD4D066CA252ABDACC10489A1917CC5073EEDF52" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7AAC2839-ABF2-4346-96AE-14DCDB318DC5}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -127,60 +127,61 @@
     <t>https://www.bis.org/doclist/reshub_papers.rss</t>
   </si>
   <si>
+    <t>https://www.hkma.gov.hk/eng/other-information/rss/rss_press-release.xml</t>
+  </si>
+  <si>
+    <t>https://www.federalreserve.gov/feeds/press_all.xml</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.fsb.org/wordpress/content_type/press/feed/</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.occ.gov/rss/occ_news.xml</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.ecb.europa.eu/rss/press.html</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.srb.europa.eu/en/rss</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.fsa.go.jp/fsaNewsListAll_rss2.xml</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.boj.or.jp/rss/whatsnew.xml</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.finma.ch/en/rss/news/</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://www.osfi-bsif.gc.ca/en/rss.xml</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>BOE1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>BOE2</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>bankofengland.co.uk/rss/publications</t>
+  </si>
+  <si>
+    <t>https://www.bankofengland.co.uk/rss/publications</t>
+  </si>
+  <si>
     <t>https://www.bankofengland.co.uk/rss/news</t>
-  </si>
-  <si>
-    <t>https://www.hkma.gov.hk/eng/other-information/rss/rss_press-release.xml</t>
-  </si>
-  <si>
-    <t>https://www.federalreserve.gov/feeds/press_all.xml</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://www.fsb.org/wordpress/content_type/press/feed/</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://www.occ.gov/rss/occ_news.xml</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://www.ecb.europa.eu/rss/press.html</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://www.srb.europa.eu/en/rss</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://www.fsa.go.jp/fsaNewsListAll_rss2.xml</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://www.boj.or.jp/rss/whatsnew.xml</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://www.finma.ch/en/rss/news/</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://www.osfi-bsif.gc.ca/en/rss.xml</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>BOE1</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>BOE2</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>bankofengland.co.uk/rss/publications</t>
-  </si>
-  <si>
-    <t>https://www.bankofengland.co.uk/rss/publications</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
@@ -534,7 +535,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -545,7 +546,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -556,7 +557,7 @@
         <v>5</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -589,7 +590,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -605,24 +606,24 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C8" t="s">
-        <v>29</v>
+      <c r="C8" s="1" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" t="s">
         <v>42</v>
-      </c>
-      <c r="C9" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -633,7 +634,7 @@
         <v>16</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -644,7 +645,7 @@
         <v>19</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -655,7 +656,7 @@
         <v>20</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -666,7 +667,7 @@
         <v>24</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -677,7 +678,7 @@
         <v>25</v>
       </c>
       <c r="C14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -688,7 +689,7 @@
         <v>26</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="5:5">
@@ -720,8 +721,9 @@
     <hyperlink ref="C13" r:id="rId21" xr:uid="{9590A641-5E0A-42AC-921B-1446080501C4}"/>
     <hyperlink ref="C15" r:id="rId22" xr:uid="{D3FF31DC-FDCF-4A6E-8617-5241B9FFE395}"/>
     <hyperlink ref="B9" r:id="rId23" display="https://www.bankofengland.co.uk/rss/publications" xr:uid="{428B6B0D-4299-47DC-A51C-997DC29E60B5}"/>
+    <hyperlink ref="C8" r:id="rId24" xr:uid="{80AF8D53-A9D0-4E6F-8EAF-4B6820D5436B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId24"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId25"/>
 </worksheet>
 </file>
</xml_diff>